<commit_message>
produktjakt: offertarket bäddar in heron (Axels krav 09-16 "det MÅSTE vara bilder i sheetet"); gemensamt ark 15/9 + 16/9 med 15 produkter; sida v22 med det arket som nedladdning
- offert.py: --fynd tar flera rundor; bilder ur korningar/<datum>/v3/bilder/ bäddas in i A:C (Pillow-tumme, 45 pt-rader); =IMAGE() bara som reserv
- Leverantorsoffert-2026-09-15-och-16.xlsx (15 rader, datum i namnet), dagens ark omskrivet med bilder

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016jBJVGuyny8S3j2XPSM26Z
</commit_message>
<xml_diff>
--- a/produktjakt/korningar/2026-09-16/Leverantorsoffert-2026-09-16.xlsx
+++ b/produktjakt/korningar/2026-09-16/Leverantorsoffert-2026-09-16.xlsx
@@ -532,6 +532,161 @@
 </styleSheet>
 </file>
 
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>4</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1600200" cy="1600200"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>8</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1600200" cy="1600200"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="2" name="Image 2" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>12</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1600200" cy="1600200"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="3" name="Image 3" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>16</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1600200" cy="1600200"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="4" name="Image 4" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>20</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1600200" cy="1600200"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="5" name="Image 5" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId5"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>24</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1600200" cy="1600200"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="6" name="Image 6" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId6"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
   <a:themeElements>
@@ -1025,7 +1180,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="24" customHeight="1" s="71">
+    <row r="5" ht="45" customHeight="1" s="71">
       <c r="A5" s="10" t="n"/>
       <c r="D5" s="18" t="inlineStr">
         <is>
@@ -1086,7 +1241,7 @@
       <c r="AT5" s="25" t="n"/>
       <c r="AU5" s="26" t="n"/>
     </row>
-    <row r="6" ht="25.5" customHeight="1" s="71">
+    <row r="6" ht="45" customHeight="1" s="71">
       <c r="D6" s="18" t="n"/>
       <c r="J6" s="15" t="n"/>
       <c r="K6" s="15" t="n"/>
@@ -1116,7 +1271,7 @@
       <c r="AR6" s="15" t="n"/>
       <c r="AS6" s="16" t="n"/>
     </row>
-    <row r="7" s="71">
+    <row r="7" ht="45" customHeight="1" s="71">
       <c r="D7" s="18" t="n"/>
       <c r="J7" s="15" t="n"/>
       <c r="K7" s="15" t="n"/>
@@ -1195,7 +1350,7 @@
       <c r="AT8" s="35" t="n"/>
       <c r="AU8" s="35" t="n"/>
     </row>
-    <row r="9" ht="24" customHeight="1" s="71">
+    <row r="9" ht="45" customHeight="1" s="71">
       <c r="A9" s="10" t="n"/>
       <c r="D9" s="18" t="inlineStr">
         <is>
@@ -1256,7 +1411,7 @@
       <c r="AT9" s="25" t="n"/>
       <c r="AU9" s="26" t="n"/>
     </row>
-    <row r="10" ht="25.5" customHeight="1" s="71">
+    <row r="10" ht="45" customHeight="1" s="71">
       <c r="D10" s="18" t="n"/>
       <c r="J10" s="15" t="n"/>
       <c r="K10" s="15" t="n"/>
@@ -1286,7 +1441,7 @@
       <c r="AR10" s="15" t="n"/>
       <c r="AS10" s="16" t="n"/>
     </row>
-    <row r="11" s="71">
+    <row r="11" ht="45" customHeight="1" s="71">
       <c r="D11" s="18" t="n"/>
       <c r="J11" s="15" t="n"/>
       <c r="K11" s="15" t="n"/>
@@ -1365,7 +1520,7 @@
       <c r="AT12" s="35" t="n"/>
       <c r="AU12" s="35" t="n"/>
     </row>
-    <row r="13" ht="24" customHeight="1" s="71">
+    <row r="13" ht="45" customHeight="1" s="71">
       <c r="A13" s="10" t="n"/>
       <c r="D13" s="18" t="inlineStr">
         <is>
@@ -1426,7 +1581,7 @@
       <c r="AT13" s="25" t="n"/>
       <c r="AU13" s="26" t="n"/>
     </row>
-    <row r="14" ht="25.5" customHeight="1" s="71">
+    <row r="14" ht="45" customHeight="1" s="71">
       <c r="D14" s="18" t="n"/>
       <c r="J14" s="15" t="n"/>
       <c r="K14" s="15" t="n"/>
@@ -1456,7 +1611,7 @@
       <c r="AR14" s="15" t="n"/>
       <c r="AS14" s="16" t="n"/>
     </row>
-    <row r="15" s="71">
+    <row r="15" ht="45" customHeight="1" s="71">
       <c r="D15" s="18" t="n"/>
       <c r="J15" s="15" t="n"/>
       <c r="K15" s="15" t="n"/>
@@ -1535,7 +1690,7 @@
       <c r="AT16" s="35" t="n"/>
       <c r="AU16" s="35" t="n"/>
     </row>
-    <row r="17" ht="24" customHeight="1" s="71">
+    <row r="17" ht="45" customHeight="1" s="71">
       <c r="A17" s="10" t="n"/>
       <c r="D17" s="18" t="inlineStr">
         <is>
@@ -1596,7 +1751,7 @@
       <c r="AT17" s="25" t="n"/>
       <c r="AU17" s="26" t="n"/>
     </row>
-    <row r="18" ht="25.5" customHeight="1" s="71">
+    <row r="18" ht="45" customHeight="1" s="71">
       <c r="D18" s="18" t="n"/>
       <c r="J18" s="15" t="n"/>
       <c r="K18" s="15" t="n"/>
@@ -1626,7 +1781,7 @@
       <c r="AR18" s="15" t="n"/>
       <c r="AS18" s="16" t="n"/>
     </row>
-    <row r="19" s="71">
+    <row r="19" ht="45" customHeight="1" s="71">
       <c r="D19" s="18" t="n"/>
       <c r="J19" s="15" t="n"/>
       <c r="K19" s="15" t="n"/>
@@ -1705,7 +1860,7 @@
       <c r="AT20" s="35" t="n"/>
       <c r="AU20" s="35" t="n"/>
     </row>
-    <row r="21" ht="24" customHeight="1" s="71">
+    <row r="21" ht="45" customHeight="1" s="71">
       <c r="A21" s="10" t="n"/>
       <c r="D21" s="18" t="inlineStr">
         <is>
@@ -1766,7 +1921,7 @@
       <c r="AT21" s="25" t="n"/>
       <c r="AU21" s="26" t="n"/>
     </row>
-    <row r="22" ht="25.5" customHeight="1" s="71">
+    <row r="22" ht="45" customHeight="1" s="71">
       <c r="D22" s="18" t="n"/>
       <c r="J22" s="15" t="n"/>
       <c r="K22" s="15" t="n"/>
@@ -1796,7 +1951,7 @@
       <c r="AR22" s="15" t="n"/>
       <c r="AS22" s="16" t="n"/>
     </row>
-    <row r="23" s="71">
+    <row r="23" ht="45" customHeight="1" s="71">
       <c r="D23" s="18" t="n"/>
       <c r="J23" s="15" t="n"/>
       <c r="K23" s="15" t="n"/>
@@ -1875,7 +2030,7 @@
       <c r="AT24" s="35" t="n"/>
       <c r="AU24" s="35" t="n"/>
     </row>
-    <row r="25" ht="24" customHeight="1" s="71">
+    <row r="25" ht="45" customHeight="1" s="71">
       <c r="A25" s="10" t="n"/>
       <c r="D25" s="18" t="inlineStr">
         <is>
@@ -1936,7 +2091,7 @@
       <c r="AT25" s="25" t="n"/>
       <c r="AU25" s="26" t="n"/>
     </row>
-    <row r="26" ht="25.5" customHeight="1" s="71">
+    <row r="26" ht="45" customHeight="1" s="71">
       <c r="D26" s="18" t="n"/>
       <c r="J26" s="15" t="n"/>
       <c r="K26" s="15" t="n"/>
@@ -1966,7 +2121,7 @@
       <c r="AR26" s="15" t="n"/>
       <c r="AS26" s="16" t="n"/>
     </row>
-    <row r="27" s="71">
+    <row r="27" ht="45" customHeight="1" s="71">
       <c r="D27" s="18" t="n"/>
       <c r="J27" s="15" t="n"/>
       <c r="K27" s="15" t="n"/>
@@ -3084,5 +3239,6 @@
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>